<commit_message>
Completed Schematic and changed spreadsheet specs
</commit_message>
<xml_diff>
--- a/ECAD/Keyboard_Teensy40_Pin_Map.xlsx
+++ b/ECAD/Keyboard_Teensy40_Pin_Map.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="254">
   <si>
     <t xml:space="preserve">Teensy 4.0 pin map - 16x6 keyboard with ST7789 display and rotary encoder</t>
   </si>
@@ -320,7 +320,7 @@
     <t xml:space="preserve">I2C_SCL</t>
   </si>
   <si>
-    <t xml:space="preserve">MCP23017 SCL (pin 12)</t>
+    <t xml:space="preserve">MCP23017 SCK/SCL (pin 12)</t>
   </si>
   <si>
     <t xml:space="preserve">A5, SCL0 (Wire), PWM</t>
@@ -452,16 +452,22 @@
     <t xml:space="preserve">Maximum key positions</t>
   </si>
   <si>
-    <t xml:space="preserve">MCP23017 I2C I/O expander - pin by pin (28-pin SPDIP / SOIC / SSOP pinout)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check the datasheet pinout if you use the QFN-28 package; its pin numbers differ.</t>
+    <t xml:space="preserve">MCP23017 - pin by pin, matched to the KiCad symbol (28-pin SPDIP / SOIC / SSOP numbering)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin names and numbers follow the symbol in the schematic. Pins 11 and 14 are NC and are not drawn on the symbol. Check the datasheet pinout if you use the QFN-28 package; its pin numbers differ.</t>
   </si>
   <si>
     <t xml:space="preserve">Chip Pin</t>
   </si>
   <si>
-    <t xml:space="preserve">Pin Name</t>
+    <t xml:space="preserve">Pin Name (on symbol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symbol Side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position on Side (left to right)</t>
   </si>
   <si>
     <t xml:space="preserve">Net / Connects To</t>
@@ -470,6 +476,9 @@
     <t xml:space="preserve">GPB0</t>
   </si>
   <si>
+    <t xml:space="preserve">Bottom</t>
+  </si>
+  <si>
     <t xml:space="preserve">COL8</t>
   </si>
   <si>
@@ -518,144 +527,168 @@
     <t xml:space="preserve">VDD</t>
   </si>
   <si>
+    <t xml:space="preserve">Right</t>
+  </si>
+  <si>
     <t xml:space="preserve">Place a 0.1 uF decoupling capacitor to GND close to this pin.</t>
   </si>
   <si>
     <t xml:space="preserve">VSS</t>
   </si>
   <si>
+    <t xml:space="preserve">Left</t>
+  </si>
+  <si>
     <t xml:space="preserve">NC</t>
   </si>
   <si>
+    <t xml:space="preserve">Not drawn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
     <t xml:space="preserve">No connect</t>
   </si>
   <si>
-    <t xml:space="preserve">Chip-select on the SPI variant (MCP23S17); unused on I2C.</t>
+    <t xml:space="preserve">Hidden on the symbol. Chip-select on the SPI variant (MCP23S17); unused on I2C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2C_SCL (Teensy 19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labeled SCK on the symbol; in I2C mode this is the SCL clock line. 2.2 kOhm pull-up to 3V3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2C_SDA (Teensy 18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hidden on the symbol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address bit 0 low.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address bit 1 low.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address bit 2 low. A0-A2 all low gives I2C address 0x20.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active low. Tie high (optionally via 10 kOhm), or drive from spare Teensy pin 21.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not needed when INT mirroring is enabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP_INT (Teensy 20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional interrupt line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPA7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST7789 1.14" 135x240 SPI display and rotary encoder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display pin order below is the common one for 8-pin modules. Vendors differ, so confirm against the silkscreen on your module.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display module (8-pin, 3.3 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teensy Pin / Rail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VCC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3 V logic and power.</t>
   </si>
   <si>
     <t xml:space="preserve">SCL</t>
   </si>
   <si>
-    <t xml:space="preserve">I2C_SCL (Teensy 19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I2C_SDA (Teensy 18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address bit 0 low.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address bit 1 low.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address bit 2 low. A0-A2 all low gives I2C address 0x20.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RESET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active low. Tie high (optionally via 10 kOhm), or drive from spare Teensy pin 21.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not needed when INT mirroring is enabled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCP_INT (Teensy 20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional interrupt line.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPA7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST7789 1.14" 135x240 SPI display and rotary encoder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Display pin order below is the common one for 8-pin modules. Vendors differ, so confirm against the silkscreen on your module.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Display module (8-pin, 3.3 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Module Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teensy Pin / Rail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VCC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.3 V logic and power.</t>
-  </si>
-  <si>
     <t xml:space="preserve">SPI clock (SCK).</t>
   </si>
   <si>
@@ -747,6 +780,9 @@
   </si>
   <si>
     <t xml:space="preserve">Pin numbers on the 'Teensy Pin Map' and 'MCP23017' sheets and the display/encoder tables are typed by hand. Column-to-MCP mapping on 'Key Matrix' is formula-driven from the Col # cells.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The MCP23017 tab follows the pin names and numbers on the KiCad symbol. The symbol labels pin 12 SCK, which is the I2C SCL clock line.</t>
   </si>
   <si>
     <t xml:space="preserve">Teensy micro-USB connector sits at the top edge of the module. Place the Teensy so that port is reachable from the case.</t>
@@ -2606,13 +2642,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2625,7 +2663,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>144</v>
       </c>
@@ -2636,6 +2674,12 @@
         <v>146</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2644,109 +2688,163 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="D5" s="5"/>
+        <v>149</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="D6" s="5"/>
+      <c r="D6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="D7" s="5"/>
+        <v>154</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D8" s="5"/>
+        <v>156</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D9" s="5"/>
+        <v>158</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D10" s="5"/>
+        <v>160</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D11" s="5"/>
+        <v>162</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="D12" s="5"/>
+        <v>164</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="C13" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>164</v>
+      <c r="F13" s="5" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2754,39 +2852,57 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>171</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>100</v>
+        <v>176</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2794,12 +2910,18 @@
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="D17" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2808,25 +2930,39 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D18" s="5"/>
+        <v>171</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="C19" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>174</v>
+      <c r="F19" s="5" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2834,13 +2970,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C20" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>176</v>
+      <c r="F20" s="5" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2848,13 +2990,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>178</v>
+      <c r="F21" s="5" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2862,13 +3010,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="C22" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>180</v>
+      <c r="F22" s="5" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2876,13 +3030,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>182</v>
+        <v>191</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2890,13 +3050,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2904,96 +3070,144 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="D25" s="5"/>
+        <v>196</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="D26" s="5"/>
+        <v>198</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D27" s="5"/>
+        <v>200</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="F27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D28" s="5"/>
+        <v>202</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="D29" s="5"/>
+        <v>204</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
         <v>26</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="D30" s="5"/>
+        <v>206</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="D31" s="5"/>
+        <v>208</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="D32" s="5"/>
+        <v>210</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="F32" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3022,17 +3236,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -3040,13 +3254,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>8</v>
@@ -3069,13 +3283,13 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>77</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3083,13 +3297,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>13</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3097,13 +3311,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>11</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3111,13 +3325,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3125,13 +3339,13 @@
         <v>6</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>9</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3139,13 +3353,13 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3153,18 +3367,18 @@
         <v>8</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3172,13 +3386,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>8</v>
@@ -3186,24 +3400,24 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>6</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>10</v>
@@ -3212,24 +3426,24 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>7</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>14</v>
@@ -3240,10 +3454,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>10</v>
@@ -3266,7 +3480,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3275,7 +3489,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3283,7 +3497,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3291,7 +3505,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3299,7 +3513,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,7 +3521,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3315,7 +3529,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3323,7 +3537,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3331,7 +3545,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3339,15 +3553,23 @@
         <v>8</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
         <v>9</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>241</v>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>